<commit_message>
chore: update news radar report 2026-07-29
</commit_message>
<xml_diff>
--- a/docs/data/rxbenefits_intel_hub_report_2026-07-29.xlsx
+++ b/docs/data/rxbenefits_intel_hub_report_2026-07-29.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,25 +446,52 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SHARx Advocates For Outcome-Driven PBM Reform Over Superficial Headlines</t>
+          <t>Wellcentra and LaborForce Media Partner to Combat Rising Employer Drug Costs</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SHARx emphasizes that current pharmacy benefit manager (PBM) reform efforts must be evaluated based on tangible financial outcomes for self-funded employers rather than legislative or media headlines. This perspective matters because employers need true cost containment and transparency rather than symbolic policy changes in the pharmacy benefits space. Key business implications include encouraging self-funded plan sponsors to look beyond surface-level PBM contract changes and demand verifiable cost-saving results from their vendor partnerships.</t>
+          <t>Wellcentra and LaborForce Media have announced a strategic partnership aimed at helping self-funded plan sponsors navigate and mitigate escalating prescription drug expenditures. This collaboration matters because employers are increasingly seeking innovative strategies to manage specialty drug inflation and overall pharmacy benefit expenses without sacrificing care quality. For businesses, this alliance highlights the growing demand for specialized consulting and educational resources that empower plan sponsors to demand greater transparency and cost containment from their pharmacy partners.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>The National Law Review</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Wed, 29 Jul 2026 10:13:06 GMT</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQekRSelBrZGNRU2RqYWdjbE01Ujg3LXpfY0VVUzdXNzctbFg0N0FTNU96c3V4aFdLWFFsX1ZSd253UFRBR0tpRkg3MWNLSmI3Tkk2bEsxWnlOSHg0aVJwR1RKcEt3TmNYdl85dFRyMTFXcmNjakRBMnRLUGJMM2RoS1FOUDV5WHlJUFBQdkV4c2FTSWgzRXNibUduNmJnbzhqNWo0d0xEamRUWjIySE4yb2RwTQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SHARx Advocates For Outcome-Driven PBM Reform Beyond Industry Headlines</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SHARx has publicly stated that true pharmacy benefit manager (PBM) reform must be evaluated based on tangible financial and clinical results rather than surface-level legislative headlines. This matters because self-funded employers continue to navigate rising specialty drug costs and complex PBM transparency issues that require genuine solutions. For RxBenefits, this emphasizes the strategic importance of demonstrating measurable cost containment and fiduciary accountability to employers seeking real value over marketing promises.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>The AI Journal</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Tue, 28 Jul 2026 12:35:17 GMT</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOeV9JcGVVcXBWSXJ6QnRKYnRpX0tncm55TmJ1dXlmd2xGUXBFU2xHWTExc0M1VEhvNjJybEFhamNFSDVQRzJmc0FSb1dlNmtLa2wyU2NGUGNmWmxnOHNqYlNzUE5JRmpPWlktUktpSlBha0FOOUtpUWJ6Nkk2cmFtWkpwSlRHQW5ybXZDeFN5dw?oc=5</t>
         </is>

</xml_diff>